<commit_message>
Ignore generated parquet artifacts and sync S1 models, strategy, and paper runner.
GitHub rejects files over 100MB; reshuffle panels and engineered features stay local. Production joblib/txt models remain tracked.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/02_research/notebooks/s1_factor_review.xlsx
+++ b/02_research/notebooks/s1_factor_review.xlsx
@@ -8,15 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\ML Algorithmic Trading\Portfolio 26\trading_portfolio\02_research\notebooks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{36FA4AC4-215C-46D9-B341-B7832CABCC9E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C653E28-7A1E-4AAF-A470-AC40A1807456}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11020" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Factors To Keep (Alphalens)" sheetId="1" r:id="rId1"/>
     <sheet name="Factors To Remove (Matrix)" sheetId="2" r:id="rId2"/>
     <sheet name="GBM Training" sheetId="3" r:id="rId3"/>
     <sheet name="Backtesting" sheetId="4" r:id="rId4"/>
+    <sheet name="Reshuffle" sheetId="5" r:id="rId5"/>
+    <sheet name="Fix Empty Tickers" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -28,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="60">
   <si>
     <t>Factors to keep</t>
   </si>
@@ -205,13 +207,82 @@
   </si>
   <si>
     <t>Linear Model</t>
+  </si>
+  <si>
+    <r>
+      <t>The baseline only trades 68 of its 100 names.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> The Ridge notebook's complete-case drop deletes any row with a NaN model feature. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>gross_profitability</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> has 36% coverage (29 tickers with zero SEC data) and </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>log_mcap</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 90% (9 tickers with zero). This is why </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>s1_linear_slim_ffill_is_predictions.parquet</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> contains 68 tickers, not 100.</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -231,6 +302,19 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
     </font>
   </fonts>
   <fills count="3">
@@ -268,7 +352,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -294,6 +378,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -884,6 +971,50 @@
     </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>131</xdr:row>
+      <xdr:rowOff>145361</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>16</xdr:col>
+      <xdr:colOff>22952</xdr:colOff>
+      <xdr:row>142</xdr:row>
+      <xdr:rowOff>154232</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="10" name="Picture 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DA2EE575-3B03-2320-DABA-9123CC02D8B8}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="0" y="24198855"/>
+          <a:ext cx="9815723" cy="2028630"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -1212,7 +1343,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F46"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="28.26953125" customWidth="1"/>
     <col min="3" max="3" width="17.6328125" customWidth="1"/>
@@ -1220,7 +1351,7 @@
     <col min="5" max="5" width="8.26953125" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1240,7 +1371,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6">
       <c r="A2" s="2" t="s">
         <v>15</v>
       </c>
@@ -1260,7 +1391,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6">
       <c r="A3" s="1" t="s">
         <v>36</v>
       </c>
@@ -1278,7 +1409,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6">
       <c r="A4" s="1" t="s">
         <v>27</v>
       </c>
@@ -1296,7 +1427,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6">
       <c r="A5" s="1" t="s">
         <v>28</v>
       </c>
@@ -1311,7 +1442,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6">
       <c r="A6" s="1" t="s">
         <v>16</v>
       </c>
@@ -1326,7 +1457,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6">
       <c r="A7" s="1" t="s">
         <v>37</v>
       </c>
@@ -1341,7 +1472,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:6">
       <c r="A8" s="1" t="s">
         <v>38</v>
       </c>
@@ -1356,7 +1487,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:6">
       <c r="A9" s="1" t="s">
         <v>39</v>
       </c>
@@ -1371,7 +1502,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:6">
       <c r="A10" s="1" t="s">
         <v>26</v>
       </c>
@@ -1386,7 +1517,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:6">
       <c r="A11" s="1" t="s">
         <v>17</v>
       </c>
@@ -1401,7 +1532,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:6">
       <c r="A12" s="1" t="s">
         <v>52</v>
       </c>
@@ -1416,7 +1547,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:6">
       <c r="A13" s="2" t="s">
         <v>14</v>
       </c>
@@ -1431,7 +1562,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:6">
       <c r="A14" s="1" t="s">
         <v>25</v>
       </c>
@@ -1446,7 +1577,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:6">
       <c r="A15" s="1" t="s">
         <v>29</v>
       </c>
@@ -1461,7 +1592,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:6">
       <c r="A16" s="1" t="s">
         <v>18</v>
       </c>
@@ -1476,7 +1607,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5">
       <c r="A17" s="1" t="s">
         <v>51</v>
       </c>
@@ -1491,7 +1622,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5">
       <c r="A18" s="2" t="s">
         <v>3</v>
       </c>
@@ -1508,7 +1639,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5">
       <c r="A19" s="2" t="s">
         <v>13</v>
       </c>
@@ -1523,7 +1654,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5">
       <c r="A20" s="2" t="s">
         <v>12</v>
       </c>
@@ -1538,7 +1669,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5">
       <c r="A21" s="1" t="s">
         <v>24</v>
       </c>
@@ -1553,7 +1684,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5">
       <c r="A22" s="2" t="s">
         <v>9</v>
       </c>
@@ -1568,7 +1699,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5">
       <c r="A23" s="1" t="s">
         <v>31</v>
       </c>
@@ -1583,7 +1714,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5">
       <c r="A24" s="1" t="s">
         <v>20</v>
       </c>
@@ -1598,7 +1729,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5">
       <c r="A25" s="1" t="s">
         <v>21</v>
       </c>
@@ -1613,7 +1744,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5">
       <c r="A26" s="2" t="s">
         <v>11</v>
       </c>
@@ -1628,7 +1759,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5">
       <c r="A27" s="1" t="s">
         <v>23</v>
       </c>
@@ -1643,7 +1774,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5">
       <c r="A28" s="2" t="s">
         <v>10</v>
       </c>
@@ -1658,7 +1789,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5">
       <c r="A29" s="1" t="s">
         <v>22</v>
       </c>
@@ -1673,7 +1804,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5">
       <c r="A30" s="1" t="s">
         <v>19</v>
       </c>
@@ -1690,7 +1821,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5">
       <c r="A31" s="1" t="s">
         <v>50</v>
       </c>
@@ -1705,7 +1836,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5">
       <c r="A32" s="1" t="s">
         <v>49</v>
       </c>
@@ -1720,7 +1851,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5">
       <c r="A33" s="1" t="s">
         <v>40</v>
       </c>
@@ -1735,7 +1866,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5">
       <c r="A34" s="1" t="s">
         <v>42</v>
       </c>
@@ -1750,7 +1881,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5">
       <c r="A35" s="1" t="s">
         <v>41</v>
       </c>
@@ -1765,7 +1896,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5">
       <c r="A36" s="1" t="s">
         <v>43</v>
       </c>
@@ -1780,7 +1911,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5">
       <c r="A37" s="1" t="s">
         <v>46</v>
       </c>
@@ -1795,7 +1926,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5">
       <c r="A38" s="1" t="s">
         <v>44</v>
       </c>
@@ -1810,7 +1941,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5">
       <c r="A39" s="1" t="s">
         <v>45</v>
       </c>
@@ -1825,7 +1956,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:5">
       <c r="A40" s="1" t="s">
         <v>47</v>
       </c>
@@ -1840,7 +1971,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:5">
       <c r="A41" s="1" t="s">
         <v>48</v>
       </c>
@@ -1855,35 +1986,35 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:5">
       <c r="A42" s="1"/>
       <c r="B42" s="1"/>
       <c r="C42" s="1"/>
       <c r="D42" s="1"/>
       <c r="E42" s="1"/>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:5">
       <c r="A43" s="1"/>
       <c r="B43" s="1"/>
       <c r="C43" s="1"/>
       <c r="D43" s="1"/>
       <c r="E43" s="1"/>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:5">
       <c r="A44" s="1"/>
       <c r="B44" s="1"/>
       <c r="C44" s="1"/>
       <c r="D44" s="1"/>
       <c r="E44" s="1"/>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:5">
       <c r="A45" s="1"/>
       <c r="B45" s="1"/>
       <c r="C45" s="1"/>
       <c r="D45" s="1"/>
       <c r="E45" s="1"/>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:5">
       <c r="A46" s="1"/>
       <c r="B46" s="1"/>
       <c r="C46" s="1"/>
@@ -1901,91 +2032,91 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CFF12DA7-1932-493E-9BFC-972882446799}">
   <dimension ref="A1:A18"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="23.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:1">
       <c r="A1" s="7" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:1">
       <c r="A2" s="5" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:1">
       <c r="A3" s="2" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:1">
       <c r="A4" s="6" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:1">
       <c r="A5" s="2" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:1">
       <c r="A6" s="2" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:1">
       <c r="A7" s="2" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:1">
       <c r="A8" s="6" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:1">
       <c r="A9" s="2" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:1">
       <c r="A10" s="2" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:1">
       <c r="A11" s="6" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:1">
       <c r="A12" s="6" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:1">
       <c r="A13" s="6" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:1">
       <c r="A14" s="6" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:1">
       <c r="A15" s="6"/>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:1">
       <c r="A16" s="6"/>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:1">
       <c r="A17" s="6"/>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:1">
       <c r="A18" s="6"/>
     </row>
   </sheetData>
@@ -2000,13 +2131,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A5BA01C-4689-4CB2-9E3B-D9376080BF6E}">
   <dimension ref="A1:C1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="51.08984375" customWidth="1"/>
     <col min="2" max="3" width="51.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3">
       <c r="A1" t="s">
         <v>56</v>
       </c>
@@ -2029,9 +2160,36 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C0BE9B27-6FD2-4F20-9949-41489FEE480F}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BFFD693-5DB6-499F-93A3-A1904BC15D10}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A283AE2-1CA0-4A4D-B460-F296D857C5BC}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.5"/>
+  <cols>
+    <col min="1" max="1" width="112.7265625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" ht="43.5">
+      <c r="A1" s="8" t="s">
+        <v>59</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>